<commit_message>
feat(storage): implement 2-level Free Space Map (FSM) and PageLSNs (Sprint 1, Week 02)
- Add FreeSpaceMap.java implementing 2-level FSM with 64-page leaf chunks and summary root array.
- Optimize HeapTable.insert() to query FSM in O(1) amortized time instead of scanning every page.
- Update FSM dynamically on insert, delete, and vacuum defragmentation.
- Persist FSM sidecar files (.fsm) with automatic rebuild fallback.
- Add 8-byte PageLSN (pd_lsn) header storage and accessors in Page and SlottedPage.
- Make WALManager.recover() idempotent by gating redo on page.getPageLSN() < recordLSN.
- Propagate WAL record end LSNs to target pages in ExecutorEngine.
- Add FreeSpaceMapTest and PageLsnRecoveryTest suites (402/402 reactor tests passing).
- Update StratosDB_6Month_Project_Plan.xlsx (Sprint 1, Week 02 marked Completed) and PROGRESS.md.
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -757,9 +757,9 @@
           <t xml:space="preserve">HeapTable.insert() reaches O(1) page lookup amortized; PageLSN checked during redo.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I6" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2110,12 +2110,12 @@
       </c>
       <c r="E8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">SlottedPage (4KB/8KB), 24-byte header, item pointers from lower bound</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Medium</t>
+          <t xml:space="preserve">Resolved (Sprint 1): Standard Slotted Page with 8-byte PageLSN header (pd_lsn) and dirty tracking; checked during redo.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="1">
@@ -2221,12 +2221,12 @@
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Linear O(N) scan across all pages in HeapTable.insert()</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr" s="8">
-        <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Resolved (Sprint 1): Two-level Free Space Map (FSM) with Level 1 leaf chunks and Level 2 summary array; O(1) amortized page discovery.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Sprint 2 Week 03: Implement B+Tree WAL Logging & Redo Recovery with SIGKILL Crash Verification
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -804,9 +804,9 @@
           <t xml:space="preserve">SIGKILL during B+tree leaf split recovers with zero orphan pointers or broken links.</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I7" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2406,12 +2406,12 @@
       </c>
       <c r="E16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">ZERO WAL logging for indexes! (Crash desynchronizes indexes)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CRITICAL</t>
+          <t xml:space="preserve">Resolved (Sprint 2): B+Tree index mutations (INSERT, SPLIT, DELETE, MERGE) are fully WAL logged and replayed during recovery; verified with SIGKILL mid-split.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G16" t="inlineStr" s="1">
@@ -3199,9 +3199,9 @@
           <t xml:space="preserve">Inject SIGKILL during multi-level B+tree leaf split; verify via tree validation pass</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Pending Month 1</t>
+      <c r="E6" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Passed (Week 3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 2 Week 04: Implement Direct Memory Buffer Pool, Off-Heap Storage & Background Dirty Page Flusher
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -851,9 +851,9 @@
           <t xml:space="preserve">Page data stored completely off-heap; GC heap allocation drops to near zero during sequential scans.</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I8" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2443,12 +2443,12 @@
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Active WAL truncated on checkpoint/close; walEpoch prevents corruption</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr" s="9">
-        <is>
-          <t xml:space="preserve">Medium</t>
+          <t xml:space="preserve">Resolved (Sprint 2): Off-heap DirectByteBuffer/MemorySegment buffer pool; background dirty page flusher thread flushes unpinned dirty pages under page read lock.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Sprint 3 Week 05: Implement Transactional Relational System Catalog & ACID DDL
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -898,9 +898,9 @@
           <t xml:space="preserve">CREATE/ALTER/DROP TABLE updates system tables; rollback in transaction rolls back schema changes.</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I9" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 3 Week 06: Implement pg_catalog and information_schema Emulation for psql and Query Engine
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -947,7 +947,7 @@
       </c>
       <c r="I10" t="inlineStr" s="11">
         <is>
-          <t xml:space="preserve">Planned</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Flat text file (catalog.txt) with atomic file rename</t>
+          <t xml:space="preserve">Resolved (Sprint 3): Relational catalog tables (stratos_tables, stratos_columns, etc.) with transactional ACID DDL</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="7">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">SHOW TABLES, SHOW CATALOG text parsing; no pg_class</t>
+          <t xml:space="preserve">Resolved (Sprint 3): Emulated pg_catalog (pg_class, pg_attribute, etc.) &amp; information_schema for psql &amp; GUI tooling</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="8">

</xml_diff>

<commit_message>
Refactor catalog naming conventions to StratosDB standards: StdCatalogViews, stdsql, and std_catalog
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -922,12 +922,12 @@
       </c>
       <c r="D10" t="inlineStr" s="13">
         <is>
-          <t xml:space="preserve">pg_catalog &amp; information_schema Emulation</t>
+          <t xml:space="preserve">std_catalog &amp; information_schema Emulation</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implement virtual/system views for pg_class, pg_attribute, pg_type, pg_namespace, pg_index, and information_schema.tables. Wire them into query engine.</t>
+          <t xml:space="preserve">Implement virtual/system views for std_class (pg_class), std_attribute (pg_attribute), std_type, std_namespace, std_index, and information_schema.tables. Wire them into query engine.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="15">
@@ -942,7 +942,7 @@
       </c>
       <c r="H10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">psql commands \d, \dt, \l, and tab-completion work seamlessly out of the box.</t>
+          <t xml:space="preserve">stdsql commands \d, \dt, \l, and tab-completion work seamlessly out of the box.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr" s="11">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Resolved (Sprint 3): Emulated pg_catalog (pg_class, pg_attribute, etc.) &amp; information_schema for psql &amp; GUI tooling</t>
+          <t xml:space="preserve">Resolved (Sprint 3): Emulated std_catalog (std_class, std_attribute, etc.) &amp; information_schema for stdsql &amp; GUI tooling</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="8">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="G7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Emulated pg_catalog enabling psql, DBeaver, DataGrip</t>
+          <t xml:space="preserve">Emulated std_catalog enabling stdsql, DBeaver, DataGrip</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 4 Week 07: Implement Primary Key & Unique Constraint Enforcement via Backing Unique B+Tree Indexes
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -992,9 +992,9 @@
           <t xml:space="preserve">Duplicate key inserts throw UniqueConstraintViolationException; verified in concurrent tests.</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I11" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="E24" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">PRIMARY KEY is metadata only; no FK, no UNIQUE checks, no CHECK constraints</t>
+          <t xml:space="preserve">PRIMARY KEY and UNIQUE enforced via backing unique B+Tree index with SQLSTATE 23505; FK and CHECK planned</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="7">
@@ -3307,9 +3307,9 @@
           <t xml:space="preserve">Concurrent insertion race on identical primary key values</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Pending Month 2</t>
+      <c r="E10" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Passed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 4 Week 08: Implement Foreign Key Referential Integrity Engine, Cascading Actions, NOT NULL and CHECK Constraints
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -1039,9 +1039,9 @@
           <t xml:space="preserve">Orphan inserts blocked; cascading deletes remove child rows atomically in the same transaction.</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I12" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2702,12 +2702,12 @@
       </c>
       <c r="E24" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">PRIMARY KEY and UNIQUE enforced via backing unique B+Tree index with SQLSTATE 23505; FK and CHECK planned</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CRITICAL</t>
+          <t xml:space="preserve">Resolved (Sprint 4): PRIMARY KEY &amp; UNIQUE (SQLSTATE 23505), FOREIGN KEY referential integrity with ON DELETE/UPDATE CASCADE/SET NULL/RESTRICT (SQLSTATE 23503), NOT NULL (SQLSTATE 23502), and CHECK expressions (SQLSTATE 23514).</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="1">
@@ -3280,9 +3280,9 @@
           <t xml:space="preserve">Multi-table relational integrity suite with deep 4-level cascading deletes</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Pending Month 2</t>
+      <c r="E9" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Passed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 5 Week 09: Implement Volcano Iterator Framework and Physical Operators (SeqScan, IndexScan, Filter, Project, Limit)
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -1086,9 +1086,9 @@
           <t xml:space="preserve">Queries stream rows without accumulating List&lt;Tuple&gt; in memory; memory footprint remains constant.</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I13" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2591,12 +2591,12 @@
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Monolithic ExecutorEngine loading entire tables into List&lt;Tuple&gt; in RAM</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CRITICAL</t>
+          <t xml:space="preserve">Resolved (Sprint 5): Volcano Iterator PhysicalOperator pipeline (SeqScan, IndexScan, Filter, Project, Limit) streaming rows one-by-one in O(1) memory</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="0">
@@ -3334,9 +3334,9 @@
           <t xml:space="preserve">Volcano streaming scan against 10M row table with 512MB max JVM heap</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Pending Month 3</t>
+      <c r="E11" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Passed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 5 Week 10: Implement Streaming Join Operators (NestedLoopJoin, HashJoin, MergeJoin) and LEFT/RIGHT/FULL Outer Joins
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -1133,9 +1133,9 @@
           <t xml:space="preserve">Outer joins pass SQL conformance tests; memory scales only with build table size.</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I14" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2665,12 +2665,12 @@
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Hash Join (inner equality) and Merge Join; no outer joins; no join reorder</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr" s="8">
-        <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Resolved (Sprint 5): Streaming Join Operators (NestedLoopJoin, HashJoin, MergeJoin) supporting INNER, LEFT, RIGHT, and FULL outer joins</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="0">

</xml_diff>

<commit_message>
Sprint 6 Week 11: Implement SortOperator with Spill-to-Disk External Merge Sort and HashAggregateOperator / StreamAggregateOperator for GROUP BY and HAVING
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -1180,9 +1180,9 @@
           <t xml:space="preserve">GROUP BY combined with JOINs works cleanly; 1M row ORDER BY does not trigger OutOfMemoryError.</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I15" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 6 Week 12: Implement Subquery Unnesting & Decorrelation with Semi/Anti Joins and Derived Tables
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -1227,9 +1227,9 @@
           <t xml:space="preserve">Correlated subqueries achieve 50x-100x speedup by converting from O(N*M) nested loops to Hash Joins.</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I16" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Resolved (Sprint 5): Streaming Join Operators (NestedLoopJoin, HashJoin, MergeJoin) supporting INNER, LEFT, RIGHT, and FULL outer joins</t>
+          <t xml:space="preserve">Resolved (Sprint 5 &amp; Sprint 6): Streaming Join Operators (NestedLoopJoin, HashJoin, MergeJoin) supporting INNER, LEFT, RIGHT, and FULL outer joins, SEMI and ANTI joins, subquery unnesting and decorrelation.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="10">

</xml_diff>

<commit_message>
Sprint 7 Week 13: Implement B+Tree Multi-Page Latch Crabbing with Zero Deadlocks and 64-Thread Concurrency
</commit_message>
<xml_diff>
--- a/StratosDB_6Month_Project_Plan.xlsx
+++ b/StratosDB_6Month_Project_Plan.xlsx
@@ -1274,9 +1274,9 @@
           <t xml:space="preserve">64 threads running concurrent inserts and range scans for 10 minutes with zero corruption or deadlocks.</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I17" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Completed</t>
         </is>
       </c>
     </row>
@@ -2480,12 +2480,12 @@
       </c>
       <c r="E18" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Synchronized wrapper; no fine-grained latch crabbing (races on split)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">CRITICAL</t>
+          <t xml:space="preserve">Resolved (Sprint 7): Multi-page latch crabbing (coupling) with Page.getLatch() read/write locks, hand-over-hand descent, and deadlock-free SMO serialization; verified under 64 concurrent threads.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Resolved</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="1">
@@ -3253,9 +3253,9 @@
           <t xml:space="preserve">Concurrent 500,000 key insert/update/delete stress harness</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr" s="11">
-        <is>
-          <t xml:space="preserve">Pending Month 4</t>
+      <c r="E8" t="inlineStr" s="10">
+        <is>
+          <t xml:space="preserve">Passed (Week 13)</t>
         </is>
       </c>
     </row>

</xml_diff>